<commit_message>
更新 2026-10-12 風險新聞明細（2026-10-16 12:32）
</commit_message>
<xml_diff>
--- a/risk_news_daily/2026-10-12.xlsx
+++ b/risk_news_daily/2026-10-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險新聞" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$O$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$Q$143</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O143"/>
+  <dimension ref="A1:Q143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,8 @@
     <col width="80" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -524,6 +526,16 @@
           <t>已人工覆核</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>曝險金額</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Event_ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -562,15 +574,13 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>破產</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>5</v>
-      </c>
+          <t>一般公司更新</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>通知、檢視授信及自營部位、持續追蹤</t>
+          <t>排除、不納入風險事件</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -589,7 +599,15 @@
         </is>
       </c>
       <c r="O2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>UBER-BANKRUPTCY-001</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -658,6 +676,14 @@
       <c r="O3" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>NTAP-DEFAULT-001</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -725,6 +751,14 @@
       <c r="O4" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>BALL-DEFAULT-001</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -792,6 +826,14 @@
       <c r="O5" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>EA-DEFAULT-001</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -859,6 +901,14 @@
       <c r="O6" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>EA-DEFAULT-001</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -926,6 +976,14 @@
       <c r="O7" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>GPN-SANCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -993,6 +1051,14 @@
       <c r="O8" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>XOM-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1060,6 +1126,14 @@
       <c r="O9" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>WMT-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1127,6 +1201,14 @@
       <c r="O10" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>COIN-REGULATORY_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1194,6 +1276,14 @@
       <c r="O11" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>UBER-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1261,6 +1351,14 @@
       <c r="O12" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>DUK-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1328,6 +1426,14 @@
       <c r="O13" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>UBER-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1395,6 +1501,14 @@
       <c r="O14" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>XOM-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1462,6 +1576,14 @@
       <c r="O15" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>XOM-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1529,6 +1651,14 @@
       <c r="O16" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>CTVA-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1596,6 +1726,14 @@
       <c r="O17" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>AXP-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1663,6 +1801,14 @@
       <c r="O18" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>SYY-REGULATORY_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1730,6 +1876,14 @@
       <c r="O19" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>XOM-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1797,6 +1951,14 @@
       <c r="O20" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>F-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1864,6 +2026,14 @@
       <c r="O21" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>T-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1931,6 +2101,14 @@
       <c r="O22" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>XOM-REGULATORY_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1998,6 +2176,14 @@
       <c r="O23" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>XOM-REGULATORY_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2065,6 +2251,14 @@
       <c r="O24" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>DUK-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2132,6 +2326,14 @@
       <c r="O25" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>CMS-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2170,15 +2372,13 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>監管裁罰</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="n">
-        <v>4</v>
-      </c>
+          <t>一般公司更新</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>通知、檢視授信及自營部位、持續追蹤</t>
+          <t>排除、不納入風險事件</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2197,7 +2397,15 @@
         </is>
       </c>
       <c r="O26" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>DUK-REGULATORY_PENALTY-001</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -2266,6 +2474,14 @@
       <c r="O27" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>DUK-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2333,6 +2549,14 @@
       <c r="O28" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>UBER-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2400,6 +2624,14 @@
       <c r="O29" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>EXPE-REGULATORY_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2467,6 +2699,14 @@
       <c r="O30" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>BKNG-REGULATORY_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2534,6 +2774,14 @@
       <c r="O31" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>MAR-REGULATORY_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2601,6 +2849,14 @@
       <c r="O32" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>XOM-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2668,6 +2924,14 @@
       <c r="O33" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2735,6 +2999,14 @@
       <c r="O34" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2802,6 +3074,14 @@
       <c r="O35" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2869,6 +3149,14 @@
       <c r="O36" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>MCD-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2936,6 +3224,14 @@
       <c r="O37" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3003,6 +3299,14 @@
       <c r="O38" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>JBHT-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3070,6 +3374,14 @@
       <c r="O39" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3137,6 +3449,14 @@
       <c r="O40" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3204,6 +3524,14 @@
       <c r="O41" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>DGX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3271,6 +3599,14 @@
       <c r="O42" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3338,6 +3674,14 @@
       <c r="O43" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>EFX-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3405,6 +3749,14 @@
       <c r="O44" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>AMZN-REGULATORY_PENALTY-001</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3472,6 +3824,14 @@
       <c r="O45" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>FSLR-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3539,6 +3899,14 @@
       <c r="O46" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>OTIS-ANTITRUST_INVESTIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3606,6 +3974,14 @@
       <c r="O47" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>PFE-MAJOR_LITIGATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3673,6 +4049,14 @@
       <c r="O48" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>NFLX-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3740,6 +4124,14 @@
       <c r="O49" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>DAL-EARNINGS_MISS-001</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3764,7 +4156,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
@@ -3806,6 +4198,14 @@
       </c>
       <c r="O50" s="2" t="b">
         <v>0</v>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>NFLX-WORKFORCE_REDUCTION-001</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -3874,6 +4274,14 @@
       <c r="O51" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>DAL-EARNINGS_MISS-001</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3941,6 +4349,14 @@
       <c r="O52" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>LITE-MAJOR_CUSTOMER_LOSS-001</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4008,6 +4424,14 @@
       <c r="O53" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>NFLX-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4075,6 +4499,14 @@
       <c r="O54" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>BA-CYBER_ATTACK-001</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4142,6 +4574,14 @@
       <c r="O55" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>PEP-OPERATING_DETERIORATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4209,6 +4649,14 @@
       <c r="O56" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>NFLX-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4276,6 +4724,14 @@
       <c r="O57" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>BLDR-OPERATING_DETERIORATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4343,6 +4799,14 @@
       <c r="O58" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>AMZN-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4410,6 +4874,14 @@
       <c r="O59" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>AMZN-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4477,6 +4949,14 @@
       <c r="O60" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>FDX-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4544,6 +5024,14 @@
       <c r="O61" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>GS-DATA_BREACH-001</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4611,6 +5099,14 @@
       <c r="O62" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>STZ-OPERATING_DETERIORATION-001</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4678,6 +5174,14 @@
       <c r="O63" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>SBUX-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4745,6 +5249,14 @@
       <c r="O64" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>AMZN-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4812,6 +5324,14 @@
       <c r="O65" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>FICO-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4879,6 +5399,14 @@
       <c r="O66" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>BA-CYBER_ATTACK-001</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4946,6 +5474,14 @@
       <c r="O67" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>UBER-SUPPLY_CHAIN_DISRUPTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5013,6 +5549,14 @@
       <c r="O68" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>MPC-EXPORT_RESTRICTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5080,6 +5624,14 @@
       <c r="O69" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>WBD-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5147,6 +5699,14 @@
       <c r="O70" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>ACN-DATA_BREACH-001</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5214,6 +5774,14 @@
       <c r="O71" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>ACN-DATA_BREACH-001</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5281,6 +5849,14 @@
       <c r="O72" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>ACN-DATA_BREACH-001</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5348,6 +5924,14 @@
       <c r="O73" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>NVDA-SUPPLY_CHAIN_DISRUPTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5415,6 +5999,14 @@
       <c r="O74" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>TTWO-CYBER_ATTACK-001</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5482,6 +6074,14 @@
       <c r="O75" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>ADM-SUPPLY_CHAIN_DISRUPTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5549,6 +6149,14 @@
       <c r="O76" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>WBD-WORKFORCE_REDUCTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5616,6 +6224,14 @@
       <c r="O77" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="2" t="inlineStr">
+        <is>
+          <t>FDX-SUPPLY_CHAIN_DISRUPTION-001</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5654,15 +6270,13 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>供應鏈中斷</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="n">
-        <v>3</v>
-      </c>
+          <t>一般公司更新</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>通知、檢視授信及自營部位、加入觀察</t>
+          <t>排除、不納入風險事件</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -5681,7 +6295,15 @@
         </is>
       </c>
       <c r="O78" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>FDX-SUPPLY_CHAIN_DISRUPTION-001</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -5750,6 +6372,14 @@
       <c r="O79" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="2" t="inlineStr">
+        <is>
+          <t>XEL-TARIFF-001</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5817,6 +6447,14 @@
       <c r="O80" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>NXPI-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5884,6 +6522,14 @@
       <c r="O81" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="2" t="inlineStr">
+        <is>
+          <t>CBOE-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5951,6 +6597,14 @@
       <c r="O82" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" s="2" t="inlineStr">
+        <is>
+          <t>CBOE-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6018,6 +6672,14 @@
       <c r="O83" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" s="2" t="inlineStr">
+        <is>
+          <t>DLTR-TARIFF-001</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6085,6 +6747,14 @@
       <c r="O84" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>ITW-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6152,6 +6822,14 @@
       <c r="O85" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" s="2" t="inlineStr">
+        <is>
+          <t>NXPI-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6219,6 +6897,14 @@
       <c r="O86" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="2" t="inlineStr">
+        <is>
+          <t>LDOS-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6286,6 +6972,14 @@
       <c r="O87" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q87" s="2" t="inlineStr">
+        <is>
+          <t>NXPI-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6353,6 +7047,14 @@
       <c r="O88" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>TYL-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6420,6 +7122,14 @@
       <c r="O89" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q89" s="2" t="inlineStr">
+        <is>
+          <t>PSX-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6487,6 +7197,14 @@
       <c r="O90" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="2" t="inlineStr">
+        <is>
+          <t>NXPI-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6554,6 +7272,14 @@
       <c r="O91" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" s="2" t="inlineStr">
+        <is>
+          <t>BLDR-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6621,6 +7347,14 @@
       <c r="O92" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>JBHT-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6688,6 +7422,14 @@
       <c r="O93" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" s="2" t="inlineStr">
+        <is>
+          <t>BLDR-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6755,6 +7497,14 @@
       <c r="O94" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q94" s="2" t="inlineStr">
+        <is>
+          <t>NKE-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6822,6 +7572,14 @@
       <c r="O95" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" s="2" t="inlineStr">
+        <is>
+          <t>BLDR-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6889,6 +7647,14 @@
       <c r="O96" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>LEN-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6956,6 +7722,14 @@
       <c r="O97" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" s="2" t="inlineStr">
+        <is>
+          <t>LDOS-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7023,6 +7797,14 @@
       <c r="O98" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P98" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q98" s="2" t="inlineStr">
+        <is>
+          <t>BLDR-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7061,15 +7843,13 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>關稅</t>
-        </is>
-      </c>
-      <c r="J99" s="2" t="n">
-        <v>2</v>
-      </c>
+          <t>一般公司更新</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr"/>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>僅紀錄</t>
+          <t>排除、不納入風險事件</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr">
@@ -7088,7 +7868,15 @@
         </is>
       </c>
       <c r="O99" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" s="2" t="inlineStr">
+        <is>
+          <t>DUK-TARIFF-001</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -7157,6 +7945,14 @@
       <c r="O100" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q100" s="2" t="inlineStr">
+        <is>
+          <t>AXP-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7224,6 +8020,14 @@
       <c r="O101" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>BLDR-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7291,6 +8095,14 @@
       <c r="O102" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q102" s="2" t="inlineStr">
+        <is>
+          <t>UAL-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7358,6 +8170,14 @@
       <c r="O103" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q103" s="2" t="inlineStr">
+        <is>
+          <t>NXPI-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7425,6 +8245,14 @@
       <c r="O104" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P104" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" s="2" t="inlineStr">
+        <is>
+          <t>BNY-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7490,7 +8318,15 @@
         </is>
       </c>
       <c r="O105" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" s="2" t="inlineStr">
+        <is>
+          <t>DLTR-ANALYST_DOWNGRADE-001</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -7557,7 +8393,15 @@
         </is>
       </c>
       <c r="O106" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" s="2" t="inlineStr">
+        <is>
+          <t>KR-ANALYST_DOWNGRADE-001</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -7626,6 +8470,14 @@
       <c r="O107" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" s="2" t="inlineStr">
+        <is>
+          <t>EIX-ANALYST_DOWNGRADE-001</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7693,6 +8545,14 @@
       <c r="O108" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" s="2" t="inlineStr">
+        <is>
+          <t>BALL-TARIFF-001</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7760,6 +8620,14 @@
       <c r="O109" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" s="2" t="inlineStr">
+        <is>
+          <t>DUK-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7827,6 +8695,14 @@
       <c r="O110" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" s="2" t="inlineStr">
+        <is>
+          <t>KR-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7894,6 +8770,14 @@
       <c r="O111" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" s="2" t="inlineStr">
+        <is>
+          <t>DUK-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7961,6 +8845,14 @@
       <c r="O112" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" s="2" t="inlineStr">
+        <is>
+          <t>AAPL-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8028,6 +8920,14 @@
       <c r="O113" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" s="2" t="inlineStr">
+        <is>
+          <t>AOS-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8095,6 +8995,14 @@
       <c r="O114" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q114" s="2" t="inlineStr">
+        <is>
+          <t>ETN-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -8162,6 +9070,14 @@
       <c r="O115" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q115" s="2" t="inlineStr">
+        <is>
+          <t>ABT-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8227,7 +9143,15 @@
         </is>
       </c>
       <c r="O116" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q116" s="2" t="inlineStr">
+        <is>
+          <t>TMUS-PRICE_MOVEMENT-001</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -8294,7 +9218,15 @@
         </is>
       </c>
       <c r="O117" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q117" s="2" t="inlineStr">
+        <is>
+          <t>T-PRICE_MOVEMENT-001</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -8363,6 +9295,14 @@
       <c r="O118" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q118" s="2" t="inlineStr">
+        <is>
+          <t>EIX-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -8430,6 +9370,14 @@
       <c r="O119" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P119" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q119" s="2" t="inlineStr">
+        <is>
+          <t>PWR-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -8497,6 +9445,14 @@
       <c r="O120" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P120" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q120" s="2" t="inlineStr">
+        <is>
+          <t>EXPD-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -8564,6 +9520,14 @@
       <c r="O121" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q121" s="2" t="inlineStr">
+        <is>
+          <t>CMCSA-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -8629,7 +9593,15 @@
         </is>
       </c>
       <c r="O122" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P122" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q122" s="2" t="inlineStr">
+        <is>
+          <t>VZ-PRICE_MOVEMENT-001</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -8696,7 +9668,15 @@
         </is>
       </c>
       <c r="O123" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q123" s="2" t="inlineStr">
+        <is>
+          <t>T-PRICE_MOVEMENT-001</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -8765,6 +9745,14 @@
       <c r="O124" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q124" s="2" t="inlineStr">
+        <is>
+          <t>UBER-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8832,6 +9820,14 @@
       <c r="O125" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q125" s="2" t="inlineStr">
+        <is>
+          <t>TMUS-PRICE_MOVEMENT-001</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -8899,6 +9895,14 @@
       <c r="O126" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q126" s="2" t="inlineStr">
+        <is>
+          <t>UBER-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8966,6 +9970,14 @@
       <c r="O127" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q127" s="2" t="inlineStr">
+        <is>
+          <t>DUK-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9033,6 +10045,14 @@
       <c r="O128" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q128" s="2" t="inlineStr">
+        <is>
+          <t>DAL-PRICE_MOVEMENT-001</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9100,6 +10120,14 @@
       <c r="O129" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q129" s="2" t="inlineStr">
+        <is>
+          <t>VZ-PRICE_MOVEMENT-001</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -9167,6 +10195,14 @@
       <c r="O130" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q130" s="2" t="inlineStr">
+        <is>
+          <t>ETR-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -9234,6 +10270,14 @@
       <c r="O131" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q131" s="2" t="inlineStr">
+        <is>
+          <t>ETR-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -9301,6 +10345,14 @@
       <c r="O132" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q132" s="2" t="inlineStr">
+        <is>
+          <t>CSX-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -9368,6 +10420,14 @@
       <c r="O133" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q133" s="2" t="inlineStr">
+        <is>
+          <t>DUK-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -9435,6 +10495,14 @@
       <c r="O134" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P134" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q134" s="2" t="inlineStr">
+        <is>
+          <t>CTVA-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -9473,34 +10541,40 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>估值疑慮</t>
-        </is>
-      </c>
-      <c r="J135" s="2" t="n">
+          <t>一般公司更新</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr"/>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>排除、不納入風險事件</t>
+        </is>
+      </c>
+      <c r="L135" s="2" t="inlineStr">
+        <is>
+          <t>overvalued</t>
+        </is>
+      </c>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOVpLWUM1MzVUM0E2UE9SWTRvaGFPcUxJTWlNa2RHNXpjWmFUQzR2SnpRNGR0OXhnYnBndW5ZUFp0Q2xidHVIejdFYzBlX25XWkMtcXQyaDV5cVR5TGF6NUNRbEdTWXlfUHlIU0tFelhPeUZ4eDlOWDN4T0ZwVTJ3NjhRcS0wZEFmWjB0RTBfbnlIeDZoUVlTeUwxTUwxQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="N135" s="2" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="O135" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="K135" s="2" t="inlineStr">
-        <is>
-          <t>僅紀錄</t>
-        </is>
-      </c>
-      <c r="L135" s="2" t="inlineStr">
-        <is>
-          <t>overvalued</t>
-        </is>
-      </c>
-      <c r="M135" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOOVpLWUM1MzVUM0E2UE9SWTRvaGFPcUxJTWlNa2RHNXpjWmFUQzR2SnpRNGR0OXhnYnBndW5ZUFp0Q2xidHVIejdFYzBlX25XWkMtcXQyaDV5cVR5TGF6NUNRbEdTWXlfUHlIU0tFelhPeUZ4eDlOWDN4T0ZwVTJ3NjhRcS0wZEFmWjB0RTBfbnlIeDZoUVlTeUwxTUwxQQ?oc=5</t>
-        </is>
-      </c>
-      <c r="N135" s="2" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="O135" s="2" t="b">
-        <v>0</v>
+      <c r="P135" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q135" s="2" t="inlineStr">
+        <is>
+          <t>NTAP-VALUATION_CONCERN-001</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -9569,6 +10643,14 @@
       <c r="O136" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q136" s="2" t="inlineStr">
+        <is>
+          <t>CBOE-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -9636,6 +10718,14 @@
       <c r="O137" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q137" s="2" t="inlineStr">
+        <is>
+          <t>IRM-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9706,6 +10796,14 @@
       </c>
       <c r="O138" s="2" t="b">
         <v>0</v>
+      </c>
+      <c r="P138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q138" s="2" t="inlineStr">
+        <is>
+          <t>NSC-VALUATION_CONCERN-001</t>
+        </is>
       </c>
     </row>
     <row r="139">
@@ -9774,6 +10872,14 @@
       <c r="O139" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q139" s="2" t="inlineStr">
+        <is>
+          <t>BLK-NATURAL_DISASTER-001</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -9841,6 +10947,14 @@
       <c r="O140" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q140" s="2" t="inlineStr">
+        <is>
+          <t>MSI-VALUATION_CONCERN-001</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -9908,6 +11022,14 @@
       <c r="O141" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q141" s="2" t="inlineStr">
+        <is>
+          <t>PTC-PRICE_MOVEMENT-001</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -9973,7 +11095,15 @@
         </is>
       </c>
       <c r="O142" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q142" s="2" t="inlineStr">
+        <is>
+          <t>STX-PRICE_MOVEMENT-001</t>
+        </is>
       </c>
     </row>
     <row r="143">
@@ -10040,11 +11170,19 @@
         </is>
       </c>
       <c r="O143" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q143" s="2" t="inlineStr">
+        <is>
+          <t>WDC-PRICE_MOVEMENT-001</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O143"/>
+  <autoFilter ref="A1:Q143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>